<commit_message>
fix: some clean up
</commit_message>
<xml_diff>
--- a/data/result.xlsx
+++ b/data/result.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>model_filters</t>
+          <t>context_filters</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -516,72 +516,72 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>response_time</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>sentence_count</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>word_count</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>avg_sentence_len</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>unique_word_ratio</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>faithfulness_score_entailment</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>faithfulness_score_neutral</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>faithfulness_score_contradiction</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>answer_correctness_literal</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>answer_correctness_neural</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>answer_relevance</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>jaccard_similarity</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>cosine_tag_answer</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>relevance</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>response_time</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/org/hse/elective_courses/MN_OI', 'file_280.docx', 'Учебный процесс', 'Траектории обучения', 'https://electives.hse.ru/', 'file_193.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Онлайн-обучение', 'Дополнительное образование', 'https://www.hse.ru/docs/289423580.html', 'file_21.docx', 'Учебный процесс', 'https://www.hse.ru/docs/490481113.html', 'file_26.docx', 'Учебный процесс', 'Траектории обучения']</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/org/hse/elective_courses/MN_OI', 'https://electives.hse', 'https://www.hse.ru/docs/289423580.html', 'https://www.hse.ru/docs/490481113.html']</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>3</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O2" t="n">
         <v>79</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" t="b">
         <v>1</v>
       </c>
       <c r="Q2" t="inlineStr">
@@ -662,46 +662,46 @@
         </is>
       </c>
       <c r="R2" t="n">
+        <v>8.412186999999999</v>
+      </c>
+      <c r="S2" t="n">
         <v>4</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>72</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>18</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>0.9166666666666666</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>0.6118826866149902</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>0.1876140832901001</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>0.2005032300949097</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>29.3062528169179</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>0.5740185379981995</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>0.3189123272895813</v>
       </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
       <c r="AC2" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="AD2" t="n">
         <v>0.3276387453079224</v>
       </c>
-      <c r="AD2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>8.412186999999999</v>
+      <c r="AE2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -742,7 +742,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'file_254.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'https://www.hse.ru/studyspravka/kontr', 'file_270.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/480101460.html', 'file_75.docx', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/552116522.html', 'file_20.docx', 'Учебный процесс']</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -760,19 +760,19 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'https://www.hse.ru/studyspravka/kontr', 'https://www.hse.ru/docs/480101460.html', 'https://www.hse.ru/docs/552116522.html']</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>3</v>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O3" t="n">
         <v>71</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" t="b">
         <v>1</v>
       </c>
       <c r="Q3" t="inlineStr">
@@ -781,46 +781,46 @@
         </is>
       </c>
       <c r="R3" t="n">
+        <v>13.259808</v>
+      </c>
+      <c r="S3" t="n">
         <v>5</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>66</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>13.2</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>0.8787878787878788</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>0.6489430069923401</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>0.1347694993019104</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>0.2162874639034271</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>27.46260354420096</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>0.6110109686851501</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>0.3152807950973511</v>
       </c>
-      <c r="AB3" t="n">
-        <v>0</v>
-      </c>
       <c r="AC3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="AD3" t="n">
         <v>0.3684489727020264</v>
       </c>
-      <c r="AD3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>13.259808</v>
+      <c r="AE3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -861,7 +861,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'file_254.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'https://electives.hse.ru/kpv', 'file_394.docx', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'https://www.hse.ru/docs/490481113.html', 'file_26.docx', 'Учебный процесс', 'Траектории обучения', 'https://www.hse.ru/studyspravka/kontr', 'file_270.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов']</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -879,19 +879,19 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'https://electives.hse', 'https://www.hse.ru/docs/490481113.html', 'https://www.hse.ru/studyspravka/kontr']</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>3</v>
       </c>
       <c r="N4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O4" t="n">
         <v>73</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" t="b">
         <v>1</v>
       </c>
       <c r="Q4" t="inlineStr">
@@ -900,46 +900,46 @@
         </is>
       </c>
       <c r="R4" t="n">
+        <v>18.527903</v>
+      </c>
+      <c r="S4" t="n">
         <v>8</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>69</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>8.625</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>0.8115942028985508</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>0.7002854347229004</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>0.218845397233963</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>0.08086920529603958</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>22.23612969715292</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>0.5656224489212036</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>0.3846144080162048</v>
       </c>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
       <c r="AC4" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="AD4" t="n">
         <v>0.3417143523693085</v>
       </c>
-      <c r="AD4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>18.527903</v>
+      <c r="AE4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -980,7 +980,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'file_254.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'https://electives.hse.ru/kpv', 'file_394.docx', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'https://www.hse.ru/docs/490481113.html', 'file_26.docx', 'Учебный процесс', 'Траектории обучения', 'https://www.hse.ru/studyspravka/kontr', 'file_270.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/studyspravka/plan', 'file_254.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'https://www.hse.ru/org/hse/elective_courses/MN_OI', 'file_280.docx', 'Учебный процесс', 'Траектории обучения', 'https://electives.hse.ru/', 'file_193.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Онлайн-обучение', 'Дополнительное образование', 'https://www.hse.ru/docs/289423580.html', 'file_21.docx', 'Учебный процесс']</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -998,19 +998,19 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'https://electives.hse', 'https://www.hse.ru/docs/490481113.html', 'https://www.hse.ru/studyspravka/kontr']</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>3</v>
       </c>
       <c r="N5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O5" t="n">
         <v>73</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" t="b">
         <v>1</v>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1019,46 +1019,46 @@
         </is>
       </c>
       <c r="R5" t="n">
+        <v>9.437844</v>
+      </c>
+      <c r="S5" t="n">
         <v>8</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>69</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>8.625</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>0.8115942028985508</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>0.7002854347229004</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>0.218845397233963</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>0.08086920529603958</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>22.23612969715292</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>0.5656224489212036</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>0.3846144080162048</v>
       </c>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
       <c r="AC5" t="n">
+        <v>0.03846153846153846</v>
+      </c>
+      <c r="AD5" t="n">
         <v>0.3417143523693085</v>
       </c>
-      <c r="AD5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>9.437844</v>
+      <c r="AE5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/lms', 'file_9.docx', 'Учебный процесс', 'Цифровые системы', 'https://www.hse.ru/studyspravka/step', 'file_555.docx', 'Деньги', 'Учебный процесс', 'Цифровые системы', 'https://www.hse.ru/evaluation/students_structure', 'file_508.docx', 'Практическая подготовка', 'Цифровые системы', 'Обратная связь', 'https://www.hse.ru/studyspravka/kursovrab', 'file_275.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Наука']</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1117,19 +1117,19 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/lms', 'https://www.hse.ru/studyspravka/step', 'https://www.hse.ru/evaluation/students_structure', 'https://www.hse.ru/studyspravka/kursovrab']</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>8</v>
       </c>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O6" t="n">
         <v>63</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" t="b">
         <v>1</v>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1138,46 +1138,46 @@
         </is>
       </c>
       <c r="R6" t="n">
+        <v>12.788267</v>
+      </c>
+      <c r="S6" t="n">
         <v>8</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>58</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>7.25</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>0.8620689655172413</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>0.5816411375999451</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>0.3026489317417145</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>0.1157098859548569</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>18.94528557621851</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>0.568882167339325</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>0.524564802646637</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.3308235108852386</v>
+      </c>
+      <c r="AE6" t="b">
         <v>0</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>0.3308235108852386</v>
-      </c>
-      <c r="AD6" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>12.788267</v>
       </c>
     </row>
     <row r="7">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/evaluation/students_mission', 'file_510.docx', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'https://www.hse.ru/studyspravka/new_regulations', 'file_367.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/studyspravka/vks', 'file_198.docx', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'https://www.hse.ru/dataculture/dc_courses', 'file_2.docx', 'Учебный процесс', 'Траектории обучения', 'Цифровые компетенции']</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1236,19 +1236,19 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/evaluation/students_mission', 'https://www.hse.ru/studyspravka/new_regulations', 'https://www.hse.ru/studyspravka/vks', 'https://www.hse.ru/dataculture/dc_courses']</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>4</v>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O7" t="n">
         <v>50</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7" t="b">
         <v>1</v>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1257,46 +1257,46 @@
         </is>
       </c>
       <c r="R7" t="n">
+        <v>16.902959</v>
+      </c>
+      <c r="S7" t="n">
         <v>7</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>43</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>6.142857142857143</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>0.9767441860465116</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>0.2970072627067566</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>0.6198377013206482</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>0.08315511047840118</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>14.65227638656207</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>0.5120701789855957</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>0.3483472466468811</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.3166845142841339</v>
+      </c>
+      <c r="AE7" t="b">
         <v>0</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0.3166845142841339</v>
-      </c>
-      <c r="AD7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>16.902959</v>
       </c>
     </row>
     <row r="8">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'file_254.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'https://www.hse.ru/studyspravka/kontr', 'file_270.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/552116522.html', 'file_20.docx', 'Учебный процесс', 'https://www.hse.ru/docs/480101460.html', 'file_75.docx', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов']</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1355,19 +1355,19 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'https://www.hse.ru/studyspravka/kontr', 'https://www.hse.ru/docs/552116522.html', 'https://www.hse.ru/docs/480101460.html']</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>3</v>
       </c>
       <c r="N8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O8" t="n">
         <v>68</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P8" t="b">
         <v>1</v>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1376,46 +1376,46 @@
         </is>
       </c>
       <c r="R8" t="n">
+        <v>22.491718</v>
+      </c>
+      <c r="S8" t="n">
         <v>4</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>63</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>15.75</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>0.9206349206349206</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>0.8035047650337219</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>0.09150311350822449</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>0.1049920693039894</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>26.14820319284076</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>0.613169252872467</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>0.3778668940067291</v>
       </c>
-      <c r="AB8" t="n">
-        <v>0</v>
-      </c>
       <c r="AC8" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="AD8" t="n">
         <v>0.4061979651451111</v>
       </c>
-      <c r="AD8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>22.491718</v>
+      <c r="AE8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'file_254.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'https://www.hse.ru/studyspravka/kontr', 'file_270.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/552116522.html', 'file_20.docx', 'Учебный процесс', 'https://www.hse.ru/docs/480101460.html', 'file_75.docx', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов']</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1474,19 +1474,19 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/plan', 'https://www.hse.ru/studyspravka/kontr', 'https://www.hse.ru/docs/552116522.html', 'https://www.hse.ru/docs/480101460.html']</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>3</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O9" t="n">
         <v>79</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" t="b">
         <v>1</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1495,46 +1495,46 @@
         </is>
       </c>
       <c r="R9" t="n">
+        <v>6.643707</v>
+      </c>
+      <c r="S9" t="n">
         <v>5</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>71</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>14.2</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>0.8732394366197183</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>0.8526800870895386</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>0.08085054904222488</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>0.06646936386823654</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>32.99265792104332</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AA9" t="n">
         <v>0.6415992379188538</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>0.3645102977752686</v>
       </c>
-      <c r="AB9" t="n">
-        <v>0</v>
-      </c>
       <c r="AC9" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="AD9" t="n">
         <v>0.3971919417381287</v>
       </c>
-      <c r="AD9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE9" t="n">
-        <v>6.643707</v>
+      <c r="AE9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/org/hse/elective_courses/MN_OI', 'file_280.docx', 'Учебный процесс', 'Траектории обучения', 'https://electives.hse.ru/', 'file_193.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Онлайн-обучение', 'Дополнительное образование', 'https://www.hse.ru/docs/289423580.html', 'file_21.docx', 'Учебный процесс', 'https://www.hse.ru/docs/490481113.html', 'file_26.docx', 'Учебный процесс', 'Траектории обучения']</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1593,19 +1593,19 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/org/hse/elective_courses/MN_OI', 'https://electives.hse', 'https://www.hse.ru/docs/289423580.html', 'https://www.hse.ru/docs/490481113.html']</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>3</v>
       </c>
       <c r="N10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O10" t="n">
         <v>92</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10" t="b">
         <v>1</v>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1614,46 +1614,46 @@
         </is>
       </c>
       <c r="R10" t="n">
+        <v>19.871674</v>
+      </c>
+      <c r="S10" t="n">
         <v>5</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>85</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>17</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>0.8823529411764706</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>0.4402622878551483</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>0.150562509894371</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>0.4091752171516418</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>28.8386335466637</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>0.5793296694755554</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>0.308877021074295</v>
       </c>
-      <c r="AB10" t="n">
-        <v>0</v>
-      </c>
       <c r="AC10" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="AD10" t="n">
         <v>0.3485716581344604</v>
       </c>
-      <c r="AD10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE10" t="n">
-        <v>19.871674</v>
+      <c r="AE10" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/dataculture/faq', 'file_7.docx', 'Учебный процесс', 'Траектории обучения', 'Цифровые компетенции', 'https://www.hse.ru/docs/941289807.html', 'file_119.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'https://www.hse.ru/studyspravka/instpaliat', 'file_257.docx', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'https://www.hse.ru/docs/480101460.html', 'file_75.docx', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов']</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1705,22 +1705,26 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cleaned context is empty, getting info from page contents in contexts: </t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/dataculture/faq', 'https://www.hse.ru/docs/941289807.html', 'https://www.hse.ru/studyspravka/instpaliat', 'https://www.hse.ru/docs/480101460.html']</t>
         </is>
       </c>
       <c r="M11" t="n">
         <v>7</v>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O11" t="n">
         <v>37</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P11" t="b">
         <v>1</v>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1729,46 +1733,46 @@
         </is>
       </c>
       <c r="R11" t="n">
+        <v>5.582061</v>
+      </c>
+      <c r="S11" t="n">
         <v>2</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>33</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>16.5</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>0.9393939393939394</v>
       </c>
-      <c r="V11" t="n">
-        <v>0.0591357909142971</v>
-      </c>
       <c r="W11" t="n">
-        <v>0.7407082915306091</v>
+        <v>0.1329716742038727</v>
       </c>
       <c r="X11" t="n">
-        <v>0.2001559287309647</v>
+        <v>0.802874743938446</v>
       </c>
       <c r="Y11" t="n">
+        <v>0.06415354460477829</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>2.86798102949914</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.3796107172966003</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.4682086408138275</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.4082683324813843</v>
+      </c>
+      <c r="AE11" t="b">
         <v>0</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0.05906565114855766</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>0.4682086408138275</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>0.4082683324813843</v>
-      </c>
-      <c r="AD11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>5.582061</v>
       </c>
     </row>
     <row r="12">
@@ -1809,7 +1813,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/indexam', 'file_342.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/studyspravka/indexam', 'file_342.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/docs/981357423.html', 'file_33.docx', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'https://www.hse.ru/docs/981357423.html', 'file_33.docx', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'https://www.hse.ru/studyspravka/perezach', 'file_244.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/studyspravka/perezach', 'file_244.docx', 'Учебный процесс', 'Английский язык']</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1820,22 +1824,26 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Cleaned context is empty, getting info from page contents in contexts: Независимый экзамен по английскому языку Вся актуальная информация об экзамене представлена на странице Центра независимой экспертизы по английскому языку Независимый экзамен по английскому языку Экзамен нацелен на проверку уровня владения английским языком и является обязательным для всех студентов бакалавриата и специалитета, кроме студентов очно-заочной формы обучения. Основной период сдачи НЭ С 4 модуля 2 курса по 3 модуль 3 курса. Возможна также сдача на более раннем периоде обучения — на 1 курсе или в 1-3 модулях 2 курса. НЭ по английскому языку Независимый экзамен по английскому языку Вся актуальная информация об экзамене представлена на странице Центра независимой экспертизы по английскому языку Независимый экзамен по английскому языку Экзамен нацелен на проверку уровня владения английским языком и является обязательным для всех студентов бакалавриата и специалитета, кроме студентов очно-заочной формы обучения. Основной период сдачи НЭ С 4 модуля 2 курса по 3 модуль 3 курса. Во</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/indexam', 'https://www.hse.ru/studyspravka/indexam', 'https://www.hse.ru/docs/981357423.html', 'https://www.hse.ru/docs/981357423.html', 'https://www.hse.ru/studyspravka/perezach', 'https://www.hse.ru/studyspravka/perezach', 'https://www.ets.org/toefl/institutions/ibt/about/how.html]', 'https://ielts.org/take-a-test/test-', 'http://www.cambridgeenglish.org/exams-and-tests/business-', 'http://www.cambridgeenglish.org/exams-and-tests/business-vantage/]', 'http://www.cambridgeenglish.org/exams/advanced/]', 'http://www.cambridgeenglish.org/exams/proficiency/]']</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>5</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O12" t="n">
         <v>134</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P12" t="b">
         <v>1</v>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1844,46 +1852,46 @@
         </is>
       </c>
       <c r="R12" t="n">
+        <v>75.47844499999999</v>
+      </c>
+      <c r="S12" t="n">
         <v>10</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>128</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>12.8</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>0.828125</v>
       </c>
-      <c r="V12" t="n">
-        <v>0.2264359444379807</v>
-      </c>
       <c r="W12" t="n">
-        <v>0.7399323582649231</v>
+        <v>0.9536458849906921</v>
       </c>
       <c r="X12" t="n">
-        <v>0.03363167867064476</v>
+        <v>0.03059844858944416</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>0.01575563102960587</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.009722703136503696</v>
+        <v>34.37434889468366</v>
       </c>
       <c r="AA12" t="n">
+        <v>0.6364415884017944</v>
+      </c>
+      <c r="AB12" t="n">
         <v>0.4295795261859894</v>
       </c>
-      <c r="AB12" t="n">
-        <v>0</v>
-      </c>
       <c r="AC12" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="AD12" t="n">
         <v>0.3264357149600983</v>
       </c>
-      <c r="AD12" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE12" t="n">
-        <v>75.47844499999999</v>
+      <c r="AE12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1924,7 +1932,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/578704961.html', 'file_68.docx', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/578704961.html', 'file_68.docx', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/594887310.html', 'file_51.docx', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/594887310.html', 'file_51.docx', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/552116522.html', 'file_20.docx', 'Учебный процесс', 'https://www.hse.ru/docs/552116522.html', 'file_20.docx', 'Учебный процесс']</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1935,22 +1943,26 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Cleaned context is empty, getting info from page contents in contexts: Декан факультета – руководитель факультета, в том числе в филиале, или руководитель ассоциированного с факультетом подразделения (школы, института, кафедры). Приложение к приказу НИУ ВШЭ от 22.03.2022 № 6.18.1-01/220322-6 УТВЕРЖДЕНЫ ученым советом НИУ ВШЭ протокол от 25.02.2022 № 02 Правила  перевода студентов бакалавриата, специалитета, магистратуры  Национального исследовательского университета «Высшая школа экономики» и студентов бакалавриата, специалитета, магистратуры других образовательных организаций в Национальный исследовательский университет «Высшая школа экономики» Москва, 2022 Используемые понятия и сокращения Правила – Правила перевода студентов бакалавриата, специалитета, магистратуры Национального исследовательского университета «Высшая школа экономики» и студентов бакалавриата, специалитета, магистратуры других образовательных организаций в Национальный исследовательский университет «Высшая школа экономики». НИУ ВШЭ, Университет – Национальный исследовательский универси</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/578704961.html', 'https://www.hse.ru/docs/578704961.html', 'https://www.hse.ru/docs/594887310.html', 'https://www.hse.ru/docs/594887310.html', 'https://www.hse.ru/docs/552116522.html', 'https://www.hse.ru/docs/552116522.html']</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>3</v>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O13" t="n">
         <v>48</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13" t="b">
         <v>0</v>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1959,46 +1971,46 @@
         </is>
       </c>
       <c r="R13" t="n">
+        <v>11.438174</v>
+      </c>
+      <c r="S13" t="n">
         <v>3</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>47</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>15.66666666666667</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>0.9361702127659575</v>
       </c>
-      <c r="V13" t="n">
-        <v>0.2270500808954239</v>
-      </c>
       <c r="W13" t="n">
-        <v>0.7659614086151123</v>
+        <v>0.3689203560352325</v>
       </c>
       <c r="X13" t="n">
-        <v>0.006988511886447668</v>
+        <v>0.5908573269844055</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>0.04022230580449104</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.04002891480922699</v>
+        <v>21.19742004626498</v>
       </c>
       <c r="AA13" t="n">
+        <v>0.5865079760551453</v>
+      </c>
+      <c r="AB13" t="n">
         <v>0.3319467902183533</v>
       </c>
-      <c r="AB13" t="n">
-        <v>0</v>
-      </c>
       <c r="AC13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AD13" t="n">
         <v>0.3266102075576782</v>
       </c>
-      <c r="AD13" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>11.438174</v>
+      <c r="AE13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2039,7 +2051,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/594887310.html', 'file_51.docx', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/594887310.html', 'file_51.docx', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/578704961.html', 'file_68.docx', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/578704961.html', 'file_68.docx', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'https://www.hse.ru/docs/229339407.html', 'file_55.docx', 'Учебный процесс', 'ГИА', 'https://www.hse.ru/docs/229339407.html', 'file_55.docx', 'Учебный процесс', 'ГИА']</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2050,22 +2062,26 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Cleaned context is empty, getting info from page contents in contexts: Менеджер программы – руководитель учебного офиса образовательной программы или менеджер, в функции которого входит сопровождение процессов, связанных с обучением студентов образовательной программы. Приложение  к приказу НИУ ВШЭ от 20.04.2022 № 6.18.1-01/200422-7 УТВЕРЖДЕНО ученым советом НИУ ВШЭ протокол от 25.03.2022 № 03 Положение об организации и проведении государственной итоговой аттестации студентов образовательных программ высшего образования – программ бакалавриата, специалитета и магистратуры Национального исследовательского университета «Высшая школа экономики» Используемые понятия и сокращения Положение – Положение об организации и проведении государственной итоговой аттестации студентов образовательных программ высшего образования – программ бакалавриата, специалитета и магистратуры Национального исследовательского университета «Высшая школа экономики».  НИУ ВШЭ – Национальный исследовательский университет «Высшая школа экономики». ГИА – государственная итоговая аттестация</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/594887310.html', 'https://www.hse.ru/docs/594887310.html', 'https://www.hse.ru/docs/578704961.html', 'https://www.hse.ru/docs/578704961.html', 'https://www.hse.ru/docs/229339407.html', 'https://www.hse.ru/docs/229339407.html']</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>4</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O14" t="n">
         <v>43</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P14" t="b">
         <v>0</v>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2074,46 +2090,46 @@
         </is>
       </c>
       <c r="R14" t="n">
+        <v>11.061041</v>
+      </c>
+      <c r="S14" t="n">
         <v>3</v>
       </c>
-      <c r="S14" t="n">
+      <c r="T14" t="n">
         <v>42</v>
       </c>
-      <c r="T14" t="n">
+      <c r="U14" t="n">
         <v>14</v>
       </c>
-      <c r="U14" t="n">
+      <c r="V14" t="n">
         <v>0.8809523809523809</v>
       </c>
-      <c r="V14" t="n">
-        <v>0.1757386028766632</v>
-      </c>
       <c r="W14" t="n">
-        <v>0.8179226517677307</v>
+        <v>0.8635555505752563</v>
       </c>
       <c r="X14" t="n">
-        <v>0.006338721141219139</v>
+        <v>0.09277147054672241</v>
       </c>
       <c r="Y14" t="n">
-        <v>0</v>
+        <v>0.04367303848266602</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.0575280599296093</v>
+        <v>26.99094547417145</v>
       </c>
       <c r="AA14" t="n">
+        <v>0.6204245686531067</v>
+      </c>
+      <c r="AB14" t="n">
         <v>0.4146169424057007</v>
       </c>
-      <c r="AB14" t="n">
-        <v>0</v>
-      </c>
       <c r="AC14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AD14" t="n">
         <v>0.3761751651763916</v>
       </c>
-      <c r="AD14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>11.061041</v>
+      <c r="AE14" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2154,7 +2170,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/896351333.html', 'file_63.docx', 'Деньги', 'Учебный процесс', 'ГИА', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'ВУЦ', 'https://www.hse.ru/docs/896351333.html', 'file_63.docx', 'Деньги', 'Учебный процесс', 'ГИА', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'ВУЦ', 'https://www.hse.ru/docs/802687500.html', 'file_47.docx', 'Учебный процесс', 'ВУЦ', 'https://www.hse.ru/docs/802687500.html', 'file_47.docx', 'Учебный процесс', 'ВУЦ']</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2165,22 +2181,26 @@
       <c r="J15" t="n">
         <v>1</v>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Cleaned context is empty, getting info from page contents in contexts: 6.2. При отчислении по обстоятельствам, не зависящим от воли сторон отчисление осуществляется в случае:         Приложение         к приказу НИУ ВШЭ         от 13.02.2024 № 6.18-01/130224-5      УТВЕРЖДЕНЫ ученым советом НИУ ВШЭ (протокол от 31.01.2024 № 02) ПОРЯДОК И ОСНОВАНИЯ  отчисления обучающихся из Национального исследовательского университета «Высшая школа экономики» 1. Общие положения 1.1. Порядок и основания отчисления обучающихся из Национального исследовательского университета «Высшая школа экономики» (далее соответственно – Порядок, НИУ ВШЭ или университет) устанавливают основания для отчисления и общие требования к процедуре прекращения образовательных отношений. 1.2. Особенности порядка отчисления отдельных категорий обучающихся могут быть установлены отдельными локальными нормативными актами университета. 1.3. При досрочном прекращении образовательных отношений между обучающимся и НИУ ВШЭ в трехдневный срок после издания приказа об отчислении, лицу, отчисленному из НИУ В</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/896351333.html', 'https://www.hse.ru/docs/896351333.html', 'https://www.hse.ru/docs/802687500.html', 'https://www.hse.ru/docs/802687500.html']</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>8</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O15" t="n">
         <v>99</v>
       </c>
-      <c r="P15" t="n">
+      <c r="P15" t="b">
         <v>1</v>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2189,46 +2209,46 @@
         </is>
       </c>
       <c r="R15" t="n">
+        <v>15.01742</v>
+      </c>
+      <c r="S15" t="n">
         <v>8</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>98</v>
       </c>
-      <c r="T15" t="n">
+      <c r="U15" t="n">
         <v>12.25</v>
       </c>
-      <c r="U15" t="n">
+      <c r="V15" t="n">
         <v>0.8571428571428571</v>
       </c>
-      <c r="V15" t="n">
-        <v>0.3169826865196228</v>
-      </c>
       <c r="W15" t="n">
-        <v>0.6322436332702637</v>
+        <v>0.5956088900566101</v>
       </c>
       <c r="X15" t="n">
-        <v>0.05077367275953293</v>
+        <v>0.2985297739505768</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>0.1058612987399101</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.02268198505043983</v>
+        <v>23.73566013812404</v>
       </c>
       <c r="AA15" t="n">
+        <v>0.5864739418029785</v>
+      </c>
+      <c r="AB15" t="n">
         <v>0.4444022476673126</v>
       </c>
-      <c r="AB15" t="n">
-        <v>0</v>
-      </c>
       <c r="AC15" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="AD15" t="n">
         <v>0.07933842390775681</v>
       </c>
-      <c r="AD15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>15.01742</v>
+      <c r="AE15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2269,7 +2289,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/indexam', 'file_342.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/studyspravka/indexam', 'file_342.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/docs/981357423.html', 'file_33.docx', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'https://www.hse.ru/docs/981357423.html', 'file_33.docx', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'https://www.hse.ru/studyspravka/perezach', 'file_244.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/studyspravka/perezach', 'file_244.docx', 'Учебный процесс', 'Английский язык']</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2287,19 +2307,19 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/indexam', 'https://www.hse.ru/studyspravka/indexam', 'https://www.hse.ru/docs/981357423.html', 'https://www.hse.ru/docs/981357423.html', 'https://www.hse.ru/studyspravka/perezach', 'https://www.hse.ru/studyspravka/perezach', 'https://www.ets.org/toefl/institutions/ibt/about/how.html]', 'https://ielts.org/take-a-test/test-', 'http://www.cambridgeenglish.org/exams-and-tests/business-', 'http://www.cambridgeenglish.org/exams-and-tests/business-vantage/]', 'http://www.cambridgeenglish.org/exams/advanced/]', 'http://www.cambridgeenglish.org/exams/proficiency/]']</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O16" t="n">
         <v>103</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P16" t="b">
         <v>1</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2308,46 +2328,46 @@
         </is>
       </c>
       <c r="R16" t="n">
+        <v>76.455904</v>
+      </c>
+      <c r="S16" t="n">
         <v>10</v>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>100</v>
       </c>
-      <c r="T16" t="n">
+      <c r="U16" t="n">
         <v>10</v>
       </c>
-      <c r="U16" t="n">
+      <c r="V16" t="n">
         <v>0.83</v>
       </c>
-      <c r="V16" t="n">
+      <c r="W16" t="n">
         <v>0.8105148077011108</v>
       </c>
-      <c r="W16" t="n">
+      <c r="X16" t="n">
         <v>0.1482192575931549</v>
       </c>
-      <c r="X16" t="n">
+      <c r="Y16" t="n">
         <v>0.04126590490341187</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Z16" t="n">
         <v>39.41558650841488</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="AA16" t="n">
         <v>0.6877592206001282</v>
       </c>
-      <c r="AA16" t="n">
+      <c r="AB16" t="n">
         <v>0.4140537679195404</v>
       </c>
-      <c r="AB16" t="n">
-        <v>0</v>
-      </c>
       <c r="AC16" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="AD16" t="n">
         <v>0.3441203832626343</v>
       </c>
-      <c r="AD16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>76.455904</v>
+      <c r="AE16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2388,7 +2408,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/981357423.html', 'file_33.docx', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'https://www.hse.ru/docs/981357423.html', 'file_33.docx', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'https://www.hse.ru/studyspravka/indexam', 'file_342.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/studyspravka/indexam', 'file_342.docx', 'Учебный процесс', 'Английский язык', 'https://www.hse.ru/docs/1043432520.html', 'file_29.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'https://www.hse.ru/docs/1043432520.html', 'file_29.docx', 'Деньги', 'Учебный процесс', 'Практическая подготовка']</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2406,19 +2426,19 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/981357423.html', 'https://www.hse.ru/docs/981357423.html', 'https://www.hse.ru/studyspravka/indexam', 'https://www.hse.ru/studyspravka/indexam', 'https://www.hse.ru/docs/1043432520.html', 'https://www.hse.ru/docs/1043432520.html']</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>4</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O17" t="n">
         <v>116</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P17" t="b">
         <v>1</v>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2427,46 +2447,46 @@
         </is>
       </c>
       <c r="R17" t="n">
+        <v>69.76844699999999</v>
+      </c>
+      <c r="S17" t="n">
         <v>11</v>
       </c>
-      <c r="S17" t="n">
+      <c r="T17" t="n">
         <v>117</v>
       </c>
-      <c r="T17" t="n">
+      <c r="U17" t="n">
         <v>10.63636363636364</v>
       </c>
-      <c r="U17" t="n">
+      <c r="V17" t="n">
         <v>0.8205128205128205</v>
       </c>
-      <c r="V17" t="n">
+      <c r="W17" t="n">
         <v>0.02551595121622086</v>
       </c>
-      <c r="W17" t="n">
+      <c r="X17" t="n">
         <v>0.0141816595569253</v>
       </c>
-      <c r="X17" t="n">
+      <c r="Y17" t="n">
         <v>0.9603023529052734</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Z17" t="n">
         <v>21.85423297472887</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="AA17" t="n">
         <v>0.5572482347488403</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AB17" t="n">
         <v>0.5388981103897095</v>
       </c>
-      <c r="AB17" t="n">
-        <v>0</v>
-      </c>
       <c r="AC17" t="n">
+        <v>0.07692307692307693</v>
+      </c>
+      <c r="AD17" t="n">
         <v>0.407770574092865</v>
       </c>
-      <c r="AD17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>69.76844699999999</v>
+      <c r="AE17" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2507,7 +2527,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/Skidki', 'file_469.docx', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'https://www.hse.ru/studyspravka/Skidki', 'file_469.docx', 'Деньги', 'Учебный процесс', 'Социальные вопросы']</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2525,19 +2545,19 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/studyspravka/Skidki', 'https://www.hse.ru/studyspravka/Skidki', 'https://admissions.hse', 'https://admissions.hse']</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>20</v>
       </c>
       <c r="N18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O18" t="n">
         <v>75</v>
       </c>
-      <c r="P18" t="n">
+      <c r="P18" t="b">
         <v>1</v>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2546,46 +2566,46 @@
         </is>
       </c>
       <c r="R18" t="n">
+        <v>40.69813</v>
+      </c>
+      <c r="S18" t="n">
         <v>7</v>
       </c>
-      <c r="S18" t="n">
+      <c r="T18" t="n">
         <v>71</v>
       </c>
-      <c r="T18" t="n">
+      <c r="U18" t="n">
         <v>10.14285714285714</v>
       </c>
-      <c r="U18" t="n">
+      <c r="V18" t="n">
         <v>0.8309859154929577</v>
       </c>
-      <c r="V18" t="n">
+      <c r="W18" t="n">
         <v>0.8117402195930481</v>
       </c>
-      <c r="W18" t="n">
+      <c r="X18" t="n">
         <v>0.1196868494153023</v>
       </c>
-      <c r="X18" t="n">
+      <c r="Y18" t="n">
         <v>0.06857291609048843</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Z18" t="n">
         <v>20.22542792199814</v>
       </c>
-      <c r="Z18" t="n">
+      <c r="AA18" t="n">
         <v>0.5709909200668335</v>
       </c>
-      <c r="AA18" t="n">
+      <c r="AB18" t="n">
         <v>0.4775540828704834</v>
       </c>
-      <c r="AB18" t="n">
-        <v>0</v>
-      </c>
       <c r="AC18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AD18" t="n">
         <v>0.2399558275938034</v>
       </c>
-      <c r="AD18" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>40.69813</v>
+      <c r="AE18" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2626,7 +2646,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/941197025.html', 'file_121.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'https://www.hse.ru/docs/941197025.html', 'file_121.docx', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'https://www.hse.ru/docs/807180592.html', 'file_117.docx', 'Деньги', 'Учебный процесс', 'https://www.hse.ru/docs/807180592.html', 'file_117.docx', 'Деньги', 'Учебный процесс']</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2644,19 +2664,19 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['https://www.hse.ru/docs/941197025.html', 'https://www.hse.ru/docs/941197025.html', 'https://www.hse.ru/docs/807180592.html', 'https://www.hse.ru/docs/807180592.html']</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>13</v>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O19" t="n">
         <v>75</v>
       </c>
-      <c r="P19" t="n">
+      <c r="P19" t="b">
         <v>1</v>
       </c>
       <c r="Q19" t="inlineStr">
@@ -2665,46 +2685,46 @@
         </is>
       </c>
       <c r="R19" t="n">
+        <v>23.960496</v>
+      </c>
+      <c r="S19" t="n">
         <v>9</v>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>73</v>
       </c>
-      <c r="T19" t="n">
+      <c r="U19" t="n">
         <v>8.111111111111111</v>
       </c>
-      <c r="U19" t="n">
+      <c r="V19" t="n">
         <v>0.9315068493150684</v>
       </c>
-      <c r="V19" t="n">
+      <c r="W19" t="n">
         <v>0.7287003397941589</v>
       </c>
-      <c r="W19" t="n">
+      <c r="X19" t="n">
         <v>0.1993875950574875</v>
       </c>
-      <c r="X19" t="n">
+      <c r="Y19" t="n">
         <v>0.07191210985183716</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="Z19" t="n">
         <v>18.49770865545586</v>
       </c>
-      <c r="Z19" t="n">
+      <c r="AA19" t="n">
         <v>0.5516259670257568</v>
       </c>
-      <c r="AA19" t="n">
+      <c r="AB19" t="n">
         <v>0.5642526745796204</v>
       </c>
-      <c r="AB19" t="n">
-        <v>0</v>
-      </c>
       <c r="AC19" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AD19" t="n">
         <v>0.2505658268928528</v>
       </c>
-      <c r="AD19" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE19" t="n">
-        <v>23.960496</v>
+      <c r="AE19" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2756,7 +2776,11 @@
       <c r="J20" t="n">
         <v>0</v>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cleaned context is empty, getting info from page contents in contexts: </t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>[]</t>
@@ -2766,55 +2790,55 @@
         <v>38</v>
       </c>
       <c r="N20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
         <v>6</v>
       </c>
-      <c r="P20" t="n">
+      <c r="P20" t="b">
         <v>0</v>
       </c>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="n">
-        <v>1</v>
+        <v>35.038818</v>
       </c>
       <c r="S20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T20" t="n">
         <v>6</v>
       </c>
       <c r="U20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="V20" t="n">
-        <v>0.0116930715739727</v>
+        <v>1</v>
       </c>
       <c r="W20" t="n">
-        <v>0.9848887920379639</v>
+        <v>0.04569604992866516</v>
       </c>
       <c r="X20" t="n">
-        <v>0.003418135223910213</v>
+        <v>0.9337512254714966</v>
       </c>
       <c r="Y20" t="n">
+        <v>0.02055267803370953</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>1.376907527616445</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.5088806748390198</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.4208573400974274</v>
+      </c>
+      <c r="AC20" t="n">
         <v>0</v>
       </c>
-      <c r="Z20" t="n">
-        <v>0.09988703578710556</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>0.4208573400974274</v>
-      </c>
-      <c r="AB20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC20" t="n">
+      <c r="AD20" t="n">
         <v>0.4935205280780792</v>
       </c>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="n">
-        <v>35.038818</v>
-      </c>
+      <c r="AE20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2865,7 +2889,11 @@
       <c r="J21" t="n">
         <v>0</v>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cleaned context is empty, getting info from page contents in contexts: </t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>[]</t>
@@ -2875,55 +2903,55 @@
         <v>12</v>
       </c>
       <c r="N21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
         <v>6</v>
       </c>
-      <c r="P21" t="n">
+      <c r="P21" t="b">
         <v>0</v>
       </c>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="n">
-        <v>1</v>
+        <v>47.734612</v>
       </c>
       <c r="S21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T21" t="n">
         <v>6</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="V21" t="n">
-        <v>0.0116930715739727</v>
+        <v>1</v>
       </c>
       <c r="W21" t="n">
-        <v>0.9848887920379639</v>
+        <v>0.04569604992866516</v>
       </c>
       <c r="X21" t="n">
-        <v>0.003418135223910213</v>
+        <v>0.9337512254714966</v>
       </c>
       <c r="Y21" t="n">
+        <v>0.02055267803370953</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>1.376907527616445</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0.5088806748390198</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.6003119945526123</v>
+      </c>
+      <c r="AC21" t="n">
         <v>0</v>
       </c>
-      <c r="Z21" t="n">
-        <v>0.09988703578710556</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>0.6003119945526123</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC21" t="n">
+      <c r="AD21" t="n">
         <v>0.6101843118667603</v>
       </c>
-      <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="n">
-        <v>47.734612</v>
-      </c>
+      <c r="AE21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>